<commit_message>
updated cohort and case names to align load shapes
</commit_message>
<xml_diff>
--- a/commercial measures/SWCR003-05 Refrig Fan Motor/SWCR003-05 Refrig Fan Motor_Ex/renamed_cohort.xlsx
+++ b/commercial measures/SWCR003-05 Refrig Fan Motor/SWCR003-05 Refrig Fan Motor_Ex/renamed_cohort.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27531"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\DEER-SWCR003-04\commercial measures\SWCR003-04 Refrig Fan Motor\SWCR003-04 Refrig Fan Motor_Ex\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\D-EPP\commercial measures\SWCR003-05 Refrig Fan Motor\SWCR003-05 Refrig Fan Motor_Ex\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CB611C7-D136-41C4-B5F9-9AA9EBEE772D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57574F2D-1B25-41E5-976F-483B0929CD89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -143,7 +143,7 @@
     <t>Ref_Storage</t>
   </si>
   <si>
-    <t>VertDisplay</t>
+    <t>ReachIn</t>
   </si>
 </sst>
 </file>
@@ -468,7 +468,7 @@
     <col min="3" max="3" width="9.5703125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="11.7109375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="11.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="40" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="43.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -515,7 +515,7 @@
       </c>
       <c r="G2" t="str">
         <f>A2&amp;"&amp;"&amp;B2&amp;"&amp;"&amp;C2&amp;"&amp;"&amp;D2&amp;"&amp;"&amp;E2&amp;"__"&amp;F2</f>
-        <v>Asm&amp;0&amp;cDXGF&amp;Ex&amp;Ref_Storage__VertDisplay</v>
+        <v>Asm&amp;0&amp;cDXGF&amp;Ex&amp;Ref_Storage__ReachIn</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -539,7 +539,7 @@
       </c>
       <c r="G3" t="str">
         <f t="shared" ref="G3:G26" si="0">A3&amp;"&amp;"&amp;B3&amp;"&amp;"&amp;C3&amp;"&amp;"&amp;D3&amp;"&amp;"&amp;E3&amp;"__"&amp;F3</f>
-        <v>ECC&amp;0&amp;cDXGF&amp;Ex&amp;Ref_Storage__VertDisplay</v>
+        <v>ECC&amp;0&amp;cDXGF&amp;Ex&amp;Ref_Storage__ReachIn</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -563,7 +563,7 @@
       </c>
       <c r="G4" t="str">
         <f t="shared" si="0"/>
-        <v>EPr&amp;0&amp;cDXGF&amp;Ex&amp;Ref_Storage__VertDisplay</v>
+        <v>EPr&amp;0&amp;cDXGF&amp;Ex&amp;Ref_Storage__ReachIn</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -587,7 +587,7 @@
       </c>
       <c r="G5" t="str">
         <f t="shared" si="0"/>
-        <v>ERC&amp;0&amp;cDXGF&amp;Ex&amp;Ref_Storage__VertDisplay</v>
+        <v>ERC&amp;0&amp;cDXGF&amp;Ex&amp;Ref_Storage__ReachIn</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -611,7 +611,7 @@
       </c>
       <c r="G6" t="str">
         <f t="shared" si="0"/>
-        <v>ESe&amp;0&amp;cDXGF&amp;Ex&amp;Ref_Storage__VertDisplay</v>
+        <v>ESe&amp;0&amp;cDXGF&amp;Ex&amp;Ref_Storage__ReachIn</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -635,7 +635,7 @@
       </c>
       <c r="G7" t="str">
         <f t="shared" si="0"/>
-        <v>EUn&amp;0&amp;cDXGF&amp;Ex&amp;Ref_Storage__VertDisplay</v>
+        <v>EUn&amp;0&amp;cDXGF&amp;Ex&amp;Ref_Storage__ReachIn</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
@@ -659,7 +659,7 @@
       </c>
       <c r="G8" t="str">
         <f t="shared" si="0"/>
-        <v>Fin&amp;0&amp;cDXGF&amp;Ex&amp;Ref_Storage__VertDisplay</v>
+        <v>Fin&amp;0&amp;cDXGF&amp;Ex&amp;Ref_Storage__ReachIn</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
@@ -683,7 +683,7 @@
       </c>
       <c r="G9" t="str">
         <f t="shared" si="0"/>
-        <v>Gro&amp;0&amp;cDXGF&amp;Ex&amp;Ref_Storage__VertDisplay</v>
+        <v>Gro&amp;0&amp;cDXGF&amp;Ex&amp;Ref_Storage__ReachIn</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
@@ -707,7 +707,7 @@
       </c>
       <c r="G10" t="str">
         <f t="shared" si="0"/>
-        <v>Hsp&amp;0&amp;cDXGF&amp;Ex&amp;Ref_Storage__VertDisplay</v>
+        <v>Hsp&amp;0&amp;cDXGF&amp;Ex&amp;Ref_Storage__ReachIn</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
@@ -731,7 +731,7 @@
       </c>
       <c r="G11" t="str">
         <f t="shared" si="0"/>
-        <v>Htl&amp;0&amp;cDXGF&amp;Ex&amp;Ref_Storage__VertDisplay</v>
+        <v>Htl&amp;0&amp;cDXGF&amp;Ex&amp;Ref_Storage__ReachIn</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
@@ -755,7 +755,7 @@
       </c>
       <c r="G12" t="str">
         <f t="shared" si="0"/>
-        <v>Lib&amp;0&amp;cDXGF&amp;Ex&amp;Ref_Storage__VertDisplay</v>
+        <v>Lib&amp;0&amp;cDXGF&amp;Ex&amp;Ref_Storage__ReachIn</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
@@ -779,7 +779,7 @@
       </c>
       <c r="G13" t="str">
         <f t="shared" si="0"/>
-        <v>MBT&amp;0&amp;cDXGF&amp;Ex&amp;Ref_Storage__VertDisplay</v>
+        <v>MBT&amp;0&amp;cDXGF&amp;Ex&amp;Ref_Storage__ReachIn</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -803,7 +803,7 @@
       </c>
       <c r="G14" t="str">
         <f t="shared" si="0"/>
-        <v>MLI&amp;0&amp;cDXGF&amp;Ex&amp;Ref_Storage__VertDisplay</v>
+        <v>MLI&amp;0&amp;cDXGF&amp;Ex&amp;Ref_Storage__ReachIn</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
@@ -827,7 +827,7 @@
       </c>
       <c r="G15" t="str">
         <f t="shared" si="0"/>
-        <v>Mtl&amp;0&amp;cDXGF&amp;Ex&amp;Ref_Storage__VertDisplay</v>
+        <v>Mtl&amp;0&amp;cDXGF&amp;Ex&amp;Ref_Storage__ReachIn</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
@@ -851,7 +851,7 @@
       </c>
       <c r="G16" t="str">
         <f t="shared" si="0"/>
-        <v>Nrs&amp;0&amp;cDXGF&amp;Ex&amp;Ref_Storage__VertDisplay</v>
+        <v>Nrs&amp;0&amp;cDXGF&amp;Ex&amp;Ref_Storage__ReachIn</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
@@ -875,7 +875,7 @@
       </c>
       <c r="G17" t="str">
         <f t="shared" si="0"/>
-        <v>OfL&amp;0&amp;cDXGF&amp;Ex&amp;Ref_Storage__VertDisplay</v>
+        <v>OfL&amp;0&amp;cDXGF&amp;Ex&amp;Ref_Storage__ReachIn</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
@@ -899,7 +899,7 @@
       </c>
       <c r="G18" t="str">
         <f t="shared" si="0"/>
-        <v>OfS&amp;0&amp;cDXGF&amp;Ex&amp;Ref_Storage__VertDisplay</v>
+        <v>OfS&amp;0&amp;cDXGF&amp;Ex&amp;Ref_Storage__ReachIn</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
@@ -923,7 +923,7 @@
       </c>
       <c r="G19" t="str">
         <f t="shared" si="0"/>
-        <v>Rel&amp;0&amp;cDXGF&amp;Ex&amp;Ref_Storage__VertDisplay</v>
+        <v>Rel&amp;0&amp;cDXGF&amp;Ex&amp;Ref_Storage__ReachIn</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
@@ -947,7 +947,7 @@
       </c>
       <c r="G20" t="str">
         <f t="shared" si="0"/>
-        <v>RFF&amp;0&amp;cDXGF&amp;Ex&amp;Ref_Storage__VertDisplay</v>
+        <v>RFF&amp;0&amp;cDXGF&amp;Ex&amp;Ref_Storage__ReachIn</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
@@ -971,7 +971,7 @@
       </c>
       <c r="G21" t="str">
         <f t="shared" si="0"/>
-        <v>RSD&amp;0&amp;cDXGF&amp;Ex&amp;Ref_Storage__VertDisplay</v>
+        <v>RSD&amp;0&amp;cDXGF&amp;Ex&amp;Ref_Storage__ReachIn</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
@@ -995,7 +995,7 @@
       </c>
       <c r="G22" t="str">
         <f t="shared" si="0"/>
-        <v>Rt3&amp;0&amp;cDXGF&amp;Ex&amp;Ref_Storage__VertDisplay</v>
+        <v>Rt3&amp;0&amp;cDXGF&amp;Ex&amp;Ref_Storage__ReachIn</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
@@ -1019,7 +1019,7 @@
       </c>
       <c r="G23" t="str">
         <f t="shared" si="0"/>
-        <v>RtL&amp;0&amp;cDXGF&amp;Ex&amp;Ref_Storage__VertDisplay</v>
+        <v>RtL&amp;0&amp;cDXGF&amp;Ex&amp;Ref_Storage__ReachIn</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
@@ -1043,7 +1043,7 @@
       </c>
       <c r="G24" t="str">
         <f t="shared" si="0"/>
-        <v>RtS&amp;0&amp;cDXGF&amp;Ex&amp;Ref_Storage__VertDisplay</v>
+        <v>RtS&amp;0&amp;cDXGF&amp;Ex&amp;Ref_Storage__ReachIn</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
@@ -1067,7 +1067,7 @@
       </c>
       <c r="G25" t="str">
         <f t="shared" si="0"/>
-        <v>SCn&amp;0&amp;cDXGF&amp;Ex&amp;Ref_Storage__VertDisplay</v>
+        <v>SCn&amp;0&amp;cDXGF&amp;Ex&amp;Ref_Storage__ReachIn</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
@@ -1091,7 +1091,7 @@
       </c>
       <c r="G26" t="str">
         <f t="shared" si="0"/>
-        <v>SUn&amp;0&amp;cDXGF&amp;Ex&amp;Ref_Storage__VertDisplay</v>
+        <v>SUn&amp;0&amp;cDXGF&amp;Ex&amp;Ref_Storage__ReachIn</v>
       </c>
     </row>
   </sheetData>

</xml_diff>